<commit_message>
Support TXT/DOCX/PDF/PPTX upload content and fix training_passing widget
</commit_message>
<xml_diff>
--- a/classification_society_training_platform.xlsx
+++ b/classification_society_training_platform.xlsx
@@ -819,7 +819,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S3"/>
+  <dimension ref="A1:S5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1036,6 +1036,126 @@
       <c r="S3" t="inlineStr">
         <is>
           <t>2026-05-19 10:16:12</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>TRN-7E329BA6</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Loadline</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Basic Survey</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Surveyor</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>STF-TRN-001</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Usama Saleem</t>
+        </is>
+      </c>
+      <c r="N4" t="n">
+        <v>75</v>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>Admin User</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>2026-05-21 16:05:46</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>2026-05-21 16:05:46</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>TRN-7967C46C</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Loadline</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Basic Survey</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Surveyor</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>STF-AEC0C852</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Usman Zafar</t>
+        </is>
+      </c>
+      <c r="N5" t="n">
+        <v>75</v>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>Admin User</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>2026-05-21 16:05:51</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>2026-05-21 16:05:51</t>
         </is>
       </c>
     </row>
@@ -1050,7 +1170,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U2"/>
+  <dimension ref="A1:U4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1244,7 +1364,183 @@
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>2026-05-19 10:16:29</t>
+          <t>2026-05-21 16:06:24</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>REC-0463B0B6</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>STF-SUR-002</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Sara Malik</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Surveyor</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>TRN-7E329BA6</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Loadline</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Not Marked</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Not Attempted</t>
+        </is>
+      </c>
+      <c r="N3" t="n">
+        <v>75</v>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>Not Issued</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="S3" t="n">
+        <v>0</v>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>Assigned by Admin.</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>2026-05-21 16:06:24</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>REC-5DA903B2</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>STF-62E701F0</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Muhammad Umair</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Surveyor</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>TRN-7E329BA6</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Loadline</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Not Marked</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Not Attempted</t>
+        </is>
+      </c>
+      <c r="N4" t="n">
+        <v>75</v>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>Not Issued</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="S4" t="n">
+        <v>0</v>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>Assigned by Admin.</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>2026-05-21 16:06:24</t>
         </is>
       </c>
     </row>
@@ -1462,7 +1758,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J10"/>
+  <dimension ref="A1:J14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1922,6 +2218,204 @@
       <c r="J10" t="inlineStr">
         <is>
           <t>Muhammad Umair assigned as Surveyor</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>LOG-AED386EA</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>2026-05-21 16:05:46</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Training Created</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>STF-ADMIN</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Admin User</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Admin</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>TRN-7E329BA6</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Success</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Trainer assigned: Usama Saleem</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>LOG-881E13CA</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>2026-05-21 16:05:51</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Training Created</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>STF-ADMIN</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Admin User</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Admin</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>TRN-7967C46C</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Success</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Trainer assigned: Usman Zafar</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>LOG-BC7B4C60</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>2026-05-21 16:06:20</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Trainee Assigned</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>STF-ADMIN</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Admin User</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Admin</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>STF-SUR-002</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>TRN-7E329BA6</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Success</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Assigned to Loadline</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>LOG-4C781FBA</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>2026-05-21 16:06:20</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Trainee Assigned</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>STF-ADMIN</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Admin User</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Admin</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>STF-62E701F0</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>TRN-7E329BA6</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Success</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Assigned to Loadline</t>
         </is>
       </c>
     </row>
@@ -2607,7 +3101,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7">
@@ -2627,7 +3121,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="9">
@@ -2657,7 +3151,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
     </row>
     <row r="12">
@@ -2668,7 +3162,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-05-19 11:11:20</t>
+          <t>2026-05-21 16:06:24</t>
         </is>
       </c>
     </row>

</xml_diff>